<commit_message>
Lots of script for creating presentation plots
</commit_message>
<xml_diff>
--- a/reductions.xlsx
+++ b/reductions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FEC02A8-8759-4DAF-95DE-23C87C3E1E09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43CB6F7B-C5B3-42A4-BF2E-D98F55B03AD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LabInital" sheetId="2" r:id="rId1"/>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="161">
   <si>
     <t>ID</t>
   </si>
@@ -2054,6 +2054,18 @@
   </si>
   <si>
     <t>Note</t>
+  </si>
+  <si>
+    <t>PSA</t>
+  </si>
+  <si>
+    <t>FSA</t>
+  </si>
+  <si>
+    <t>Final Accumulated Emission (% TAN)</t>
+  </si>
+  <si>
+    <t>valve</t>
   </si>
 </sst>
 </file>
@@ -2158,7 +2170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -2197,6 +2209,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4105,7 +4120,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.88671875" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" customWidth="1"/>
     <col min="6" max="6" width="11.33203125" customWidth="1"/>
     <col min="9" max="9" width="10.88671875" customWidth="1"/>
     <col min="12" max="12" width="11.5546875" customWidth="1"/>
@@ -4120,7 +4135,7 @@
         <v>110</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
       <c r="D1" s="21" t="s">
         <v>144</v>
@@ -4221,11 +4236,11 @@
         <v>14.670999999999999</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F7" si="0">$L$2-C3</f>
+        <f>$L$2-C3</f>
         <v>15.751666666666669</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I7" si="1">(1-C3/$L$2)*100</f>
+        <f>(1-C3/$L$2)*100</f>
         <v>51.776088004558005</v>
       </c>
       <c r="L3">
@@ -4247,21 +4262,21 @@
       <c r="B4" s="17">
         <v>25</v>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="24">
         <v>30.72</v>
       </c>
       <c r="F4">
-        <f t="shared" si="0"/>
+        <f>$L$2-C4</f>
         <v>-0.29733333333333078</v>
       </c>
       <c r="I4">
-        <f t="shared" si="1"/>
+        <f>(1-C4/$L$2)*100</f>
         <v>-0.9773414559319793</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
-        <v>102</v>
+        <v>158</v>
       </c>
       <c r="B5" s="17">
         <v>3</v>
@@ -4278,7 +4293,7 @@
         <v>3.8517425782220762</v>
       </c>
       <c r="F5">
-        <f t="shared" si="0"/>
+        <f>$L$2-C5</f>
         <v>23.271666666666668</v>
       </c>
       <c r="G5" s="5">
@@ -4289,7 +4304,7 @@
         <v>8.4</v>
       </c>
       <c r="I5">
-        <f t="shared" si="1"/>
+        <f>(1-C5/$L$2)*100</f>
         <v>76.494499715124689</v>
       </c>
       <c r="J5" s="5">
@@ -4303,7 +4318,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
-        <v>102</v>
+        <v>158</v>
       </c>
       <c r="B6" s="17">
         <v>8</v>
@@ -4312,17 +4327,17 @@
         <v>11.129</v>
       </c>
       <c r="F6">
-        <f t="shared" si="0"/>
+        <f>$L$2-C6</f>
         <v>19.293666666666667</v>
       </c>
       <c r="I6">
-        <f t="shared" si="1"/>
+        <f>(1-C6/$L$2)*100</f>
         <v>63.41872288206163</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
-        <v>102</v>
+        <v>158</v>
       </c>
       <c r="B7" s="17">
         <v>24</v>
@@ -4331,11 +4346,11 @@
         <v>16.548999999999999</v>
       </c>
       <c r="F7">
-        <f t="shared" si="0"/>
+        <f>$L$2-C7</f>
         <v>13.873666666666669</v>
       </c>
       <c r="I7">
-        <f t="shared" si="1"/>
+        <f>(1-C7/$L$2)*100</f>
         <v>45.603059122584042</v>
       </c>
     </row>
@@ -4440,11 +4455,11 @@
         <v>16.167999999999999</v>
       </c>
       <c r="F12">
-        <f t="shared" ref="F12:F16" si="2">$L$3-C12</f>
+        <f>$L$3-C12</f>
         <v>8.0940000000000012</v>
       </c>
       <c r="I12">
-        <f t="shared" ref="I12:I16" si="3">(1-C12/$L$3)*100</f>
+        <f>(1-C12/$L$3)*100</f>
         <v>33.360811145000412</v>
       </c>
     </row>
@@ -4459,22 +4474,22 @@
         <v>15.208</v>
       </c>
       <c r="F13">
-        <f t="shared" si="2"/>
+        <f>$L$3-C13</f>
         <v>9.0540000000000003</v>
       </c>
       <c r="I13">
-        <f t="shared" si="3"/>
+        <f>(1-C13/$L$3)*100</f>
         <v>37.317616025059763</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="23" t="s">
-        <v>104</v>
+        <v>157</v>
       </c>
       <c r="B14" s="17">
         <v>4</v>
       </c>
-      <c r="C14" s="17">
+      <c r="C14" s="24">
         <v>6.0149999999999997</v>
       </c>
       <c r="D14">
@@ -4486,7 +4501,7 @@
         <v>5.448634650585003</v>
       </c>
       <c r="F14">
-        <f t="shared" si="2"/>
+        <f>$L$3-C14</f>
         <v>18.247</v>
       </c>
       <c r="G14" s="5">
@@ -4498,7 +4513,7 @@
         <v>5.4486346505850056</v>
       </c>
       <c r="I14">
-        <f t="shared" si="3"/>
+        <f>(1-C14/$L$3)*100</f>
         <v>75.208144423378116</v>
       </c>
       <c r="J14" s="5">
@@ -4512,7 +4527,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="23" t="s">
-        <v>104</v>
+        <v>157</v>
       </c>
       <c r="B15" s="17">
         <v>20</v>
@@ -4521,17 +4536,17 @@
         <v>17.387</v>
       </c>
       <c r="F15">
-        <f t="shared" si="2"/>
+        <f>$L$3-C15</f>
         <v>6.875</v>
       </c>
       <c r="I15">
-        <f t="shared" si="3"/>
+        <f>(1-C15/$L$3)*100</f>
         <v>28.336493281675047</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="23" t="s">
-        <v>104</v>
+        <v>157</v>
       </c>
       <c r="B16" s="17">
         <v>23</v>
@@ -4540,11 +4555,11 @@
         <v>17.751000000000001</v>
       </c>
       <c r="F16">
-        <f t="shared" si="2"/>
+        <f>$L$3-C16</f>
         <v>6.5109999999999992</v>
       </c>
       <c r="I16">
-        <f t="shared" si="3"/>
+        <f>(1-C16/$L$3)*100</f>
         <v>26.836204764652539</v>
       </c>
     </row>
@@ -4890,7 +4905,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{159F5624-4B84-4AAD-81A6-879EEC15CB26}">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" customWidth="1"/>
@@ -4902,225 +4917,255 @@
     <col min="10" max="10" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:13" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B1" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="C1" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>151</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>152</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="F1" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="G1" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="H1" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="I1" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="J1" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="J1" s="21" t="s">
+      <c r="K1" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="K1" s="21" t="s">
+      <c r="L1" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="L1" s="21" t="s">
+      <c r="M1" s="21" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>4</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="17">
+      <c r="C2" s="17">
         <v>10.289</v>
       </c>
-      <c r="C2" s="5">
-        <f>AVERAGE(B2:B4)</f>
+      <c r="D2" s="5">
+        <f>AVERAGE(C2:C4)</f>
         <v>9.870333333333333</v>
       </c>
-      <c r="D2" s="5">
-        <f>_xlfn.STDEV.P(B2:B4)</f>
+      <c r="E2" s="5">
+        <f>_xlfn.STDEV.P(C2:C4)</f>
         <v>1.5705163340620134</v>
       </c>
-      <c r="E2" s="5">
-        <f t="shared" ref="E2:E7" si="0">ABS(B2-$K$2)</f>
+      <c r="F2" s="5">
+        <f>ABS(C2-$L$2)</f>
         <v>5.1220000000000017</v>
       </c>
-      <c r="F2" s="5">
-        <f>AVERAGE(E2:E4)</f>
+      <c r="G2" s="5">
+        <f>AVERAGE(F2:F4)</f>
         <v>5.5406666666666675</v>
       </c>
-      <c r="G2" s="5">
-        <f>_xlfn.STDEV.P(E2:E4)</f>
+      <c r="H2" s="5">
+        <f>_xlfn.STDEV.P(F2:F4)</f>
         <v>1.5705163340620054</v>
       </c>
-      <c r="H2">
-        <f>(1-(B2/$K$2))*100</f>
+      <c r="I2">
+        <f>(1-(C2/$L$2))*100</f>
         <v>33.236000259554878</v>
       </c>
-      <c r="I2" s="5">
-        <f>AVERAGE(H2:H4)</f>
+      <c r="J2" s="5">
+        <f>AVERAGE(I2:I4)</f>
         <v>35.952674496571717</v>
       </c>
-      <c r="J2" s="5">
-        <f>_xlfn.STDEV.P(H2:H4)</f>
+      <c r="K2" s="5">
+        <f>_xlfn.STDEV.P(I2:I4)</f>
         <v>10.190878814236624</v>
       </c>
-      <c r="K2" s="5">
-        <f>AVERAGE(B8:B10)</f>
+      <c r="L2" s="5">
+        <f>AVERAGE(C8:C10)</f>
         <v>15.411000000000001</v>
       </c>
-      <c r="L2" s="5">
-        <f>_xlfn.STDEV.P(B8:B10)</f>
+      <c r="M2" s="5">
+        <f>_xlfn.STDEV.P(C8:C10)</f>
         <v>0.66911932169581478</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="17" t="s">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>14</v>
+      </c>
+      <c r="B3" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="B3" s="17">
+      <c r="C3" s="17">
         <v>11.55</v>
       </c>
-      <c r="E3" s="5">
-        <f t="shared" si="0"/>
+      <c r="F3" s="5">
+        <f>ABS(C3-$L$2)</f>
         <v>3.8610000000000007</v>
       </c>
-      <c r="H3">
-        <f t="shared" ref="H3:H7" si="1">(1-(B3/$K$2))*100</f>
+      <c r="I3">
+        <f>(1-(C3/$L$2))*100</f>
         <v>25.053533190578158</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="17" t="s">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>17</v>
+      </c>
+      <c r="B4" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="B4" s="17">
+      <c r="C4" s="17">
         <v>7.7720000000000002</v>
       </c>
-      <c r="E4" s="5">
-        <f t="shared" si="0"/>
+      <c r="F4" s="5">
+        <f>ABS(C4-$L$2)</f>
         <v>7.6390000000000011</v>
       </c>
-      <c r="H4">
-        <f t="shared" si="1"/>
+      <c r="I4">
+        <f>(1-(C4/$L$2))*100</f>
         <v>49.568490039582123</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>8</v>
+      </c>
+      <c r="B5" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="17">
+      <c r="C5" s="17">
         <v>7.1459999999999999</v>
       </c>
-      <c r="C5" s="5">
-        <f>AVERAGE(B5:B7)</f>
+      <c r="D5" s="5">
+        <f>AVERAGE(C5:C7)</f>
         <v>9.870333333333333</v>
       </c>
-      <c r="D5" s="5">
-        <f>_xlfn.STDEV.P(B5:B7)</f>
+      <c r="E5" s="5">
+        <f>_xlfn.STDEV.P(C5:C7)</f>
         <v>1.9375696689983146</v>
       </c>
-      <c r="E5" s="5">
-        <f t="shared" si="0"/>
+      <c r="F5" s="5">
+        <f>ABS(C5-$L$2)</f>
         <v>8.2650000000000006</v>
       </c>
-      <c r="F5" s="5">
-        <f>(AVERAGE(E5:E7))</f>
+      <c r="G5" s="5">
+        <f>(AVERAGE(F5:F7))</f>
         <v>5.5406666666666675</v>
       </c>
-      <c r="G5" s="5">
-        <f>_xlfn.STDEV.P(E5:E7)</f>
+      <c r="H5" s="5">
+        <f>_xlfn.STDEV.P(F5:F7)</f>
         <v>1.9375696689983082</v>
       </c>
-      <c r="H5">
-        <f t="shared" si="1"/>
+      <c r="I5">
+        <f>(1-(C5/$L$2))*100</f>
         <v>53.630523651936933</v>
       </c>
-      <c r="I5" s="5">
-        <f>AVERAGE(H5:H7)</f>
+      <c r="J5" s="5">
+        <f>AVERAGE(I5:I7)</f>
         <v>35.952674496571724</v>
       </c>
-      <c r="J5" s="5">
-        <f>_xlfn.STDEV.P(H5:H7)</f>
+      <c r="K5" s="5">
+        <f>_xlfn.STDEV.P(I5:I7)</f>
         <v>12.572640769569198</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>12</v>
+      </c>
+      <c r="B6" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="B6" s="17">
+      <c r="C6" s="17">
         <v>11.487</v>
       </c>
-      <c r="E6" s="5">
-        <f t="shared" si="0"/>
+      <c r="F6" s="5">
+        <f>ABS(C6-$L$2)</f>
         <v>3.9240000000000013</v>
       </c>
-      <c r="H6">
-        <f t="shared" si="1"/>
+      <c r="I6">
+        <f>(1-(C6/$L$2))*100</f>
         <v>25.462332100447739</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="17" t="s">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>18</v>
+      </c>
+      <c r="B7" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="B7" s="17">
+      <c r="C7" s="17">
         <v>10.978</v>
       </c>
-      <c r="E7" s="5">
-        <f t="shared" si="0"/>
+      <c r="F7" s="5">
+        <f>ABS(C7-$L$2)</f>
         <v>4.4330000000000016</v>
       </c>
-      <c r="H7">
-        <f t="shared" si="1"/>
+      <c r="I7">
+        <f>(1-(C7/$L$2))*100</f>
         <v>28.765167737330486</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" s="17" t="s">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>11</v>
+      </c>
+      <c r="B8" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="B8" s="17">
+      <c r="C8" s="17">
         <v>14.592000000000001</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="17"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A9" s="17" t="s">
+      <c r="D8" s="5"/>
+      <c r="E8" s="17"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>13</v>
+      </c>
+      <c r="B9" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="B9" s="17">
+      <c r="C9" s="17">
         <v>16.231000000000002</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="17"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A10" s="17" t="s">
+      <c r="D9" s="5"/>
+      <c r="E9" s="17"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>15</v>
+      </c>
+      <c r="B10" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="B10" s="17">
+      <c r="C10" s="22">
         <v>15.41</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="17"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5129,228 +5174,258 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D6F3082-212A-4C06-84C5-42D2586C1A2A}">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:13" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B1" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="C1" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>151</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>152</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="F1" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="G1" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="H1" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="I1" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="J1" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="J1" s="21" t="s">
+      <c r="K1" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="K1" s="21" t="s">
+      <c r="L1" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="L1" s="21" t="s">
+      <c r="M1" s="21" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>4</v>
+      </c>
+      <c r="B2" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="B2" s="17">
+      <c r="C2" s="17">
         <v>10.294</v>
       </c>
-      <c r="C2" s="5">
-        <f>AVERAGE(B2:B4)</f>
+      <c r="D2" s="5">
+        <f>AVERAGE(C2:C4)</f>
         <v>9.9123333333333346</v>
       </c>
-      <c r="D2" s="5">
-        <f>_xlfn.STDEV.P(B2:B4)</f>
+      <c r="E2" s="5">
+        <f>_xlfn.STDEV.P(C2:C4)</f>
         <v>1.6619916432468045</v>
       </c>
-      <c r="E2" s="5">
-        <f t="shared" ref="E2:E7" si="0">ABS(B2-$K$2)</f>
+      <c r="F2" s="5">
+        <f>ABS(C2-$L$2)</f>
         <v>6.7076666666666647</v>
       </c>
-      <c r="F2" s="5">
-        <f>AVERAGE(E2:E4)</f>
+      <c r="G2" s="5">
+        <f>AVERAGE(F2:F4)</f>
         <v>7.0893333333333315</v>
       </c>
-      <c r="G2" s="5">
-        <f>_xlfn.STDEV.P(E2:E4)</f>
+      <c r="H2" s="5">
+        <f>_xlfn.STDEV.P(F2:F4)</f>
         <v>1.6619916432468085</v>
       </c>
-      <c r="H2">
-        <f>(1-(B2/$K$2))*100</f>
+      <c r="I2">
+        <f>(1-(C2/$L$2))*100</f>
         <v>39.452994804430929</v>
       </c>
-      <c r="I2" s="5">
-        <f>AVERAGE(H2:H4)</f>
+      <c r="J2" s="5">
+        <f>AVERAGE(I2:I4)</f>
         <v>41.697872757572775</v>
       </c>
-      <c r="J2" s="5">
-        <f>_xlfn.STDEV.P(H2:H4)</f>
+      <c r="K2" s="5">
+        <f>_xlfn.STDEV.P(I2:I4)</f>
         <v>9.7754630521329702</v>
       </c>
-      <c r="K2" s="7">
-        <f>AVERAGE(B8:B10)</f>
+      <c r="L2" s="7">
+        <f>AVERAGE(C8:C10)</f>
         <v>17.001666666666665</v>
       </c>
-      <c r="L2" s="5">
-        <f>_xlfn.STDEV.P(B8:B10)</f>
+      <c r="M2" s="5">
+        <f>_xlfn.STDEV.P(C8:C10)</f>
         <v>1.0608629610945155</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="17" t="s">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>14</v>
+      </c>
+      <c r="B3" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="B3" s="22">
+      <c r="C3" s="22">
         <v>11.73</v>
       </c>
-      <c r="E3" s="5">
-        <f t="shared" si="0"/>
+      <c r="F3" s="5">
+        <f>ABS(C3-$L$2)</f>
         <v>5.2716666666666647</v>
       </c>
-      <c r="H3">
-        <f t="shared" ref="H3:H7" si="1">(1-(B3/$K$2))*100</f>
+      <c r="I3">
+        <f>(1-(C3/$L$2))*100</f>
         <v>31.006764042740897</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="17" t="s">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>17</v>
+      </c>
+      <c r="B4" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="B4" s="17">
+      <c r="C4" s="17">
         <v>7.7130000000000001</v>
       </c>
-      <c r="E4" s="5">
-        <f t="shared" si="0"/>
+      <c r="F4" s="5">
+        <f>ABS(C4-$L$2)</f>
         <v>9.2886666666666642</v>
       </c>
-      <c r="H4">
-        <f t="shared" si="1"/>
+      <c r="I4">
+        <f>(1-(C4/$L$2))*100</f>
         <v>54.633859425546504</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>8</v>
+      </c>
+      <c r="B5" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="17">
+      <c r="C5" s="17">
         <v>7.2069999999999999</v>
       </c>
-      <c r="C5" s="5">
-        <f>AVERAGE(B5:B7)</f>
+      <c r="D5" s="5">
+        <f>AVERAGE(C5:C7)</f>
         <v>10.052333333333332</v>
       </c>
-      <c r="D5" s="5">
-        <f>_xlfn.STDEV.P(B5:B7)</f>
+      <c r="E5" s="5">
+        <f>_xlfn.STDEV.P(C5:C7)</f>
         <v>2.0245357218110271</v>
       </c>
-      <c r="E5" s="5">
-        <f t="shared" si="0"/>
+      <c r="F5" s="5">
+        <f>ABS(C5-$L$2)</f>
         <v>9.7946666666666644</v>
       </c>
-      <c r="F5" s="5">
-        <f>(AVERAGE(E5:E7))</f>
+      <c r="G5" s="5">
+        <f>(AVERAGE(F5:F7))</f>
         <v>6.9493333333333318</v>
       </c>
-      <c r="G5" s="5">
-        <f>_xlfn.STDEV.P(E5:E7)</f>
+      <c r="H5" s="5">
+        <f>_xlfn.STDEV.P(F5:F7)</f>
         <v>2.024535721811024</v>
       </c>
-      <c r="H5">
-        <f t="shared" si="1"/>
+      <c r="I5">
+        <f>(1-(C5/$L$2))*100</f>
         <v>57.610038231545921</v>
       </c>
-      <c r="I5" s="5">
-        <f>AVERAGE(H5:H7)</f>
+      <c r="J5" s="5">
+        <f>AVERAGE(I5:I7)</f>
         <v>40.874424076070973</v>
       </c>
-      <c r="J5" s="5">
-        <f>_xlfn.STDEV.P(H5:H7)</f>
+      <c r="K5" s="5">
+        <f>_xlfn.STDEV.P(I5:I7)</f>
         <v>11.907866219847213</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>12</v>
+      </c>
+      <c r="B6" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="B6" s="17">
+      <c r="C6" s="17">
         <v>11.750999999999999</v>
       </c>
-      <c r="E6" s="5">
-        <f t="shared" si="0"/>
+      <c r="F6" s="5">
+        <f>ABS(C6-$L$2)</f>
         <v>5.2506666666666657</v>
       </c>
-      <c r="H6">
-        <f t="shared" si="1"/>
+      <c r="I6">
+        <f>(1-(C6/$L$2))*100</f>
         <v>30.883246740515634</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="17" t="s">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>18</v>
+      </c>
+      <c r="B7" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="B7" s="17">
+      <c r="C7" s="17">
         <v>11.199</v>
       </c>
-      <c r="E7" s="5">
-        <f t="shared" si="0"/>
+      <c r="F7" s="5">
+        <f>ABS(C7-$L$2)</f>
         <v>5.8026666666666653</v>
       </c>
-      <c r="H7">
-        <f t="shared" si="1"/>
+      <c r="I7">
+        <f>(1-(C7/$L$2))*100</f>
         <v>34.129987256151352</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A8" s="17" t="s">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>11</v>
+      </c>
+      <c r="B8" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="B8" s="17">
+      <c r="C8" s="17">
         <v>15.789</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="17"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A9" s="17" t="s">
+      <c r="D8" s="5"/>
+      <c r="E8" s="17"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>13</v>
+      </c>
+      <c r="B9" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="B9" s="17">
+      <c r="C9" s="17">
         <v>18.373000000000001</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="17"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A10" s="17" t="s">
+      <c r="D9" s="5"/>
+      <c r="E9" s="17"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>15</v>
+      </c>
+      <c r="B10" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="B10" s="17">
+      <c r="C10" s="17">
         <v>16.843</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="17"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>